<commit_message>
new data chnra 1
</commit_message>
<xml_diff>
--- a/nachr_db_manual.xlsx
+++ b/nachr_db_manual.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F71BF2B-5FA5-4765-BE7F-28DDFEFA497D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D651CB2-E718-401C-BE05-08A0F54C629D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23205" yWindow="7320" windowWidth="17925" windowHeight="9825" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2235" yWindow="1695" windowWidth="24585" windowHeight="12945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$7</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="28">
   <si>
     <t>OID</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t>no-net-effect</t>
+  </si>
+  <si>
+    <t>DOI</t>
   </si>
 </sst>
 </file>
@@ -455,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
@@ -465,11 +468,11 @@
     <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
     <col min="10" max="10" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,8 +509,11 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -542,7 +548,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -577,7 +583,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -612,7 +618,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -647,7 +653,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -682,7 +688,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -717,11 +723,11 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="I8" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M7" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>